<commit_message>
2026-03-05 NHL Scoreboard Streamlit Version, GamePredictions
</commit_message>
<xml_diff>
--- a/Python/Thingiverse/model_stats.xlsx
+++ b/Python/Thingiverse/model_stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Thingiverse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11AB1550-20FB-413E-ABD0-78257F1A5803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E9C4E2-ABA6-4FBC-85D3-9AA6DE276AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{AA65E66E-25AF-41FC-AF3D-E4037625FDAB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>Mammoth</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>QMJHL</t>
-  </si>
-  <si>
-    <t>Team</t>
   </si>
   <si>
     <t>Views</t>
@@ -111,7 +108,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>tat</t>
+    <t>Model</t>
   </si>
 </sst>
 </file>
@@ -119,7 +116,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -155,41 +152,41 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -211,14 +208,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V19" totalsRowShown="0">
-  <autoFilter ref="A1:V19" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V25" totalsRowShown="0">
+  <autoFilter ref="A1:V25" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
   <tableColumns count="22">
     <tableColumn id="22" xr3:uid="{B838C6CD-92E8-4070-81DB-2EDE900509A2}" name="Date"/>
-    <tableColumn id="1" xr3:uid="{C06BFB11-D5FB-45F8-853C-B38F6CA36FF6}" name="Team"/>
+    <tableColumn id="1" xr3:uid="{C06BFB11-D5FB-45F8-853C-B38F6CA36FF6}" name="Model"/>
     <tableColumn id="13" xr3:uid="{AEE26F58-911F-4534-94C6-8FCA31D6F4B1}" name="Published"/>
     <tableColumn id="14" xr3:uid="{11FE9DF7-F747-41F2-BE31-8FAB66C0B838}" name="Age" dataDxfId="11">
-      <calculatedColumnFormula>NOW()-Table1[[#This Row],[Published]]</calculatedColumnFormula>
+      <calculatedColumnFormula>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{7E393A08-4718-4CB8-8F50-8ACBD51A470F}" name="Views" dataDxfId="10"/>
     <tableColumn id="3" xr3:uid="{AE7E7C79-96E4-4AA4-8ABE-36217F4A6424}" name="Downloads"/>
@@ -560,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC85C3B-1FD4-46FE-8A2F-07E281673B93}">
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
@@ -589,70 +586,70 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
         <v>27</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" t="s">
-        <v>13</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="P1" s="4" t="s">
+      <c r="R1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="T1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="T1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="V1" s="4" t="s">
-        <v>26</v>
       </c>
       <c r="W1"/>
     </row>
@@ -667,8 +664,8 @@
         <v>45784</v>
       </c>
       <c r="D2" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>291.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>278</v>
       </c>
       <c r="E2" s="3">
         <v>658</v>
@@ -707,28 +704,28 @@
         <v>7.5987841945288756E-3</v>
       </c>
       <c r="P2" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>2.2560862281528107</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.3669064748201438</v>
       </c>
       <c r="Q2" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.49030445383868076</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.51438848920863312</v>
       </c>
       <c r="R2" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>3.7715727218360057E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.9568345323741004E-2</v>
       </c>
       <c r="S2" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
-        <v>1.7143512371981844E-2</v>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7985611510791366E-2</v>
       </c>
       <c r="T2" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>997</v>
       </c>
       <c r="U2" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>3.41841636697318</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.5863309352517985</v>
       </c>
       <c r="V2" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -747,8 +744,8 @@
         <v>45785</v>
       </c>
       <c r="D3" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>290.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>277</v>
       </c>
       <c r="E3" s="3">
         <v>307</v>
@@ -787,19 +784,19 @@
         <v>0</v>
       </c>
       <c r="P3" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.056233168919499</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.1083032490974729</v>
       </c>
       <c r="Q3" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.27523991372495088</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.28880866425992779</v>
       </c>
       <c r="R3" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>1.3761995686247546E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>1.444043321299639E-2</v>
       </c>
       <c r="S3" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T3" s="4">
@@ -807,8 +804,8 @@
         <v>479</v>
       </c>
       <c r="U3" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>1.6479989834281437</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7292418772563176</v>
       </c>
       <c r="V3" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -827,8 +824,8 @@
         <v>45930</v>
       </c>
       <c r="D4" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>145.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>132</v>
       </c>
       <c r="E4" s="3">
         <v>206</v>
@@ -867,19 +864,19 @@
         <v>0</v>
       </c>
       <c r="P4" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.4142958761658759</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.5606060606060606</v>
       </c>
       <c r="Q4" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.56983765884353255</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.62878787878787878</v>
       </c>
       <c r="R4" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>3.4327569809851355E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.787878787878788E-2</v>
       </c>
       <c r="S4" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T4" s="4">
@@ -887,8 +884,8 @@
         <v>387</v>
       </c>
       <c r="U4" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>2.6569539032824947</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.9318181818181817</v>
       </c>
       <c r="V4" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -901,14 +898,14 @@
         <v>46062</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>45750</v>
       </c>
       <c r="D5" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>325.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>312</v>
       </c>
       <c r="E5" s="3">
         <v>150</v>
@@ -947,28 +944,28 @@
         <v>6.6666666666666671E-3</v>
       </c>
       <c r="P5" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>0.46060942070267502</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.48076923076923078</v>
       </c>
       <c r="Q5" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>7.676823678377917E-2</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.0128205128205135E-2</v>
       </c>
       <c r="R5" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>6.1414589427023335E-3</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.41025641025641E-3</v>
       </c>
       <c r="S5" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
-        <v>3.0707294713511668E-3</v>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>3.205128205128205E-3</v>
       </c>
       <c r="T5" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>210</v>
       </c>
       <c r="U5" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>0.644853188983745</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.67307692307692313</v>
       </c>
       <c r="V5" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -987,8 +984,8 @@
         <v>45932</v>
       </c>
       <c r="D6" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>143.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>130</v>
       </c>
       <c r="E6" s="3">
         <v>97</v>
@@ -1027,19 +1024,19 @@
         <v>0</v>
       </c>
       <c r="P6" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>0.67522640696006697</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.74615384615384617</v>
       </c>
       <c r="Q6" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>7.6572066768667388E-2</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.461538461538462E-2</v>
       </c>
       <c r="R6" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>6.9610969789697628E-3</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>7.6923076923076927E-3</v>
       </c>
       <c r="S6" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T6" s="4">
@@ -1047,8 +1044,8 @@
         <v>122</v>
       </c>
       <c r="U6" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>0.8492538314343111</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.93846153846153846</v>
       </c>
       <c r="V6" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1067,8 +1064,8 @@
         <v>46034</v>
       </c>
       <c r="D7" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>41.655519097221259</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>28</v>
       </c>
       <c r="E7" s="3">
         <v>79</v>
@@ -1107,19 +1104,19 @@
         <v>0</v>
       </c>
       <c r="P7" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.8965073947492808</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.8214285714285716</v>
       </c>
       <c r="Q7" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.57615414524028785</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.8571428571428571</v>
       </c>
       <c r="R7" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>4.8012845436690654E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="S7" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T7" s="4">
@@ -1127,8 +1124,8 @@
         <v>133</v>
       </c>
       <c r="U7" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>3.1928542215399283</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>4.75</v>
       </c>
       <c r="V7" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1147,8 +1144,8 @@
         <v>45784</v>
       </c>
       <c r="D8" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>291.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>283</v>
       </c>
       <c r="E8" s="3">
         <v>688</v>
@@ -1187,28 +1184,28 @@
         <v>7.2674418604651162E-3</v>
       </c>
       <c r="P8" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>2.3589473023847018</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.431095406360424</v>
       </c>
       <c r="Q8" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.50059056126186985</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.51590106007067138</v>
       </c>
       <c r="R8" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>4.1144429692756432E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>4.2402826855123678E-2</v>
       </c>
       <c r="S8" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
-        <v>1.7143512371981844E-2</v>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7667844522968199E-2</v>
       </c>
       <c r="T8" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>1036</v>
       </c>
       <c r="U8" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>3.5521357634746384</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.6607773851590104</v>
       </c>
       <c r="V8" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1226,8 +1223,8 @@
         <v>45785</v>
       </c>
       <c r="D9" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>290.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>282</v>
       </c>
       <c r="E9" s="3">
         <v>310</v>
@@ -1266,19 +1263,19 @@
         <v>0</v>
       </c>
       <c r="P9" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.0665546656841847</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.0992907801418439</v>
       </c>
       <c r="Q9" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.27523991372495088</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.28368794326241137</v>
       </c>
       <c r="R9" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>1.3761995686247546E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>1.4184397163120567E-2</v>
       </c>
       <c r="S9" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T9" s="4">
@@ -1286,8 +1283,8 @@
         <v>482</v>
       </c>
       <c r="U9" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>1.6583204801928293</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7092198581560283</v>
       </c>
       <c r="V9" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1305,8 +1302,8 @@
         <v>45930</v>
       </c>
       <c r="D10" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>145.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>137</v>
       </c>
       <c r="E10" s="3">
         <v>207</v>
@@ -1345,19 +1342,19 @@
         <v>0</v>
       </c>
       <c r="P10" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.4211613901278461</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.5109489051094891</v>
       </c>
       <c r="Q10" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.57670317280550276</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.61313868613138689</v>
       </c>
       <c r="R10" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>3.4327569809851355E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.6496350364963501E-2</v>
       </c>
       <c r="S10" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T10" s="4">
@@ -1365,8 +1362,8 @@
         <v>390</v>
       </c>
       <c r="U10" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>2.6775504451684058</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.8467153284671531</v>
       </c>
       <c r="V10" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1378,14 +1375,14 @@
         <v>46067</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1">
         <v>45750</v>
       </c>
       <c r="D11" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>325.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>317</v>
       </c>
       <c r="E11" s="3">
         <v>153</v>
@@ -1424,28 +1421,28 @@
         <v>6.5359477124183009E-3</v>
       </c>
       <c r="P11" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>0.46982160911672849</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.48264984227129337</v>
       </c>
       <c r="Q11" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>7.9838966255130331E-2</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.2018927444794956E-2</v>
       </c>
       <c r="R11" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>6.1414589427023335E-3</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.3091482649842269E-3</v>
       </c>
       <c r="S11" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
-        <v>3.0707294713511668E-3</v>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>3.1545741324921135E-3</v>
       </c>
       <c r="T11" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>215</v>
       </c>
       <c r="U11" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>0.66020683634050081</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.67823343848580442</v>
       </c>
       <c r="V11" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1463,8 +1460,8 @@
         <v>45932</v>
       </c>
       <c r="D12" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>143.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>135</v>
       </c>
       <c r="E12" s="3">
         <v>105</v>
@@ -1503,19 +1500,19 @@
         <v>0</v>
       </c>
       <c r="P12" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>0.7309151827918251</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.77777777777777779</v>
       </c>
       <c r="Q12" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>7.6572066768667388E-2</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.1481481481481488E-2</v>
       </c>
       <c r="R12" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>6.9610969789697628E-3</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>7.4074074074074077E-3</v>
       </c>
       <c r="S12" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T12" s="4">
@@ -1523,8 +1520,8 @@
         <v>130</v>
       </c>
       <c r="U12" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>0.90494260726606923</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.96296296296296291</v>
       </c>
       <c r="V12" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1542,8 +1539,8 @@
         <v>46034</v>
       </c>
       <c r="D13" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>41.655519097221259</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>33</v>
       </c>
       <c r="E13" s="3">
         <v>80</v>
@@ -1582,27 +1579,28 @@
         <v>0</v>
       </c>
       <c r="P13" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.9205138174676262</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.4242424242424243</v>
       </c>
       <c r="Q13" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.57615414524028785</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.72727272727272729</v>
       </c>
       <c r="R13" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>4.8012845436690654E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.0606060606060608E-2</v>
       </c>
       <c r="S13" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T13" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>134</v>
       </c>
-      <c r="U13" s="4" t="s">
-        <v>28</v>
+      <c r="U13" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>4.0606060606060606</v>
       </c>
       <c r="V13" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1620,8 +1618,8 @@
         <v>45784</v>
       </c>
       <c r="D14" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>291.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>291</v>
       </c>
       <c r="E14" s="3">
         <v>677</v>
@@ -1660,28 +1658,28 @@
         <v>7.385524372230428E-3</v>
       </c>
       <c r="P14" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>2.3212315751663417</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.3264604810996565</v>
       </c>
       <c r="Q14" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.51773407363385171</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.51890034364261173</v>
       </c>
       <c r="R14" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>4.1144429692756432E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>4.1237113402061855E-2</v>
       </c>
       <c r="S14" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
-        <v>1.7143512371981844E-2</v>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7182130584192441E-2</v>
       </c>
       <c r="T14" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>1035</v>
       </c>
       <c r="U14" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>3.548707061000242</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.5567010309278349</v>
       </c>
       <c r="V14" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1699,8 +1697,8 @@
         <v>45785</v>
       </c>
       <c r="D15" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>290.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>290</v>
       </c>
       <c r="E15" s="3">
         <v>316</v>
@@ -1739,19 +1737,19 @@
         <v>0</v>
       </c>
       <c r="P15" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.0871976592135562</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.0896551724137931</v>
       </c>
       <c r="Q15" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.28212091156807467</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.28275862068965518</v>
       </c>
       <c r="R15" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>1.3761995686247546E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>1.3793103448275862E-2</v>
       </c>
       <c r="S15" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T15" s="4">
@@ -1759,8 +1757,8 @@
         <v>492</v>
       </c>
       <c r="U15" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>1.6927254694084481</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.6965517241379311</v>
       </c>
       <c r="V15" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1778,8 +1776,8 @@
         <v>45930</v>
       </c>
       <c r="D16" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>145.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>145</v>
       </c>
       <c r="E16" s="3">
         <v>217</v>
@@ -1818,19 +1816,19 @@
         <v>0</v>
       </c>
       <c r="P16" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>1.4898165297475487</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.4965517241379311</v>
       </c>
       <c r="Q16" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.60416522865338385</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.60689655172413792</v>
       </c>
       <c r="R16" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>3.4327569809851355E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.4482758620689655E-2</v>
       </c>
       <c r="S16" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T16" s="4">
@@ -1838,8 +1836,8 @@
         <v>408</v>
       </c>
       <c r="U16" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>2.8011296964838706</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.8137931034482757</v>
       </c>
       <c r="V16" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1851,14 +1849,14 @@
         <v>46075</v>
       </c>
       <c r="B17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C17" s="1">
         <v>45750</v>
       </c>
       <c r="D17" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>325.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>325</v>
       </c>
       <c r="E17" s="3">
         <v>154</v>
@@ -1897,28 +1895,28 @@
         <v>6.4935064935064939E-3</v>
       </c>
       <c r="P17" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>0.47289233858807966</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.47384615384615386</v>
       </c>
       <c r="Q17" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>8.2909695726481505E-2</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.3076923076923076E-2</v>
       </c>
       <c r="R17" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>6.1414589427023335E-3</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.1538461538461538E-3</v>
       </c>
       <c r="S17" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
-        <v>3.0707294713511668E-3</v>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>3.0769230769230769E-3</v>
       </c>
       <c r="T17" s="4">
         <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
         <v>218</v>
       </c>
       <c r="U17" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>0.66941902475455428</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.67076923076923078</v>
       </c>
       <c r="V17" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -1936,8 +1934,8 @@
         <v>45932</v>
       </c>
       <c r="D18" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>143.65551909722126</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>143</v>
       </c>
       <c r="E18" s="3">
         <v>116</v>
@@ -1976,19 +1974,19 @@
         <v>0</v>
       </c>
       <c r="P18" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>0.80748724956049256</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.81118881118881114</v>
       </c>
       <c r="Q18" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>7.6572066768667388E-2</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>7.6923076923076927E-2</v>
       </c>
       <c r="R18" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>6.9610969789697628E-3</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.993006993006993E-3</v>
       </c>
       <c r="S18" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T18" s="4">
@@ -1996,8 +1994,8 @@
         <v>141</v>
       </c>
       <c r="U18" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>0.98151467403473658</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.98601398601398604</v>
       </c>
       <c r="V18" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
@@ -2015,8 +2013,8 @@
         <v>46034</v>
       </c>
       <c r="D19" s="2">
-        <f ca="1">NOW()-Table1[[#This Row],[Published]]</f>
-        <v>41.655519097221259</v>
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>41</v>
       </c>
       <c r="E19" s="3">
         <v>85</v>
@@ -2055,19 +2053,19 @@
         <v>0</v>
       </c>
       <c r="P19" s="4">
-        <f ca="1">Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
-        <v>2.0405459310593526</v>
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.0731707317073171</v>
       </c>
       <c r="Q19" s="4">
-        <f ca="1">Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
-        <v>0.57615414524028785</v>
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.58536585365853655</v>
       </c>
       <c r="R19" s="4">
-        <f ca="1">Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
-        <v>4.8012845436690654E-2</v>
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>4.878048780487805E-2</v>
       </c>
       <c r="S19" s="4">
-        <f ca="1">Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
         <v>0</v>
       </c>
       <c r="T19" s="4">
@@ -2075,16 +2073,562 @@
         <v>139</v>
       </c>
       <c r="U19" s="4">
-        <f ca="1">Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
-        <v>3.3368927578500003</v>
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.3902439024390243</v>
       </c>
       <c r="V19" s="4">
         <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
         <v>1.6352941176470588</v>
       </c>
     </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" s="1">
+        <v>45784</v>
+      </c>
+      <c r="D20" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>297</v>
+      </c>
+      <c r="E20" s="3">
+        <v>693</v>
+      </c>
+      <c r="F20">
+        <v>158</v>
+      </c>
+      <c r="G20">
+        <v>12</v>
+      </c>
+      <c r="H20">
+        <v>5</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.227994227994228</v>
+      </c>
+      <c r="N20" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.7316017316017316E-2</v>
+      </c>
+      <c r="O20" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>7.215007215007215E-3</v>
+      </c>
+      <c r="P20" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.3333333333333335</v>
+      </c>
+      <c r="Q20" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.53198653198653201</v>
+      </c>
+      <c r="R20" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>4.0404040404040407E-2</v>
+      </c>
+      <c r="S20" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.6835016835016835E-2</v>
+      </c>
+      <c r="T20" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>1065</v>
+      </c>
+      <c r="U20" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.5858585858585861</v>
+      </c>
+      <c r="V20" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.5367965367965368</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="1">
+        <v>45785</v>
+      </c>
+      <c r="D21" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>296</v>
+      </c>
+      <c r="E21" s="3">
+        <v>328</v>
+      </c>
+      <c r="F21">
+        <v>85</v>
+      </c>
+      <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.25914634146341464</v>
+      </c>
+      <c r="N21" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.2195121951219513E-2</v>
+      </c>
+      <c r="O21" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P21" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.1081081081081081</v>
+      </c>
+      <c r="Q21" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.28716216216216217</v>
+      </c>
+      <c r="R21" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>1.3513513513513514E-2</v>
+      </c>
+      <c r="S21" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T21" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>510</v>
+      </c>
+      <c r="U21" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.722972972972973</v>
+      </c>
+      <c r="V21" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.5548780487804879</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22" s="1">
+        <v>45930</v>
+      </c>
+      <c r="D22" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>151</v>
+      </c>
+      <c r="E22" s="3">
+        <v>226</v>
+      </c>
+      <c r="F22">
+        <v>100</v>
+      </c>
+      <c r="G22">
+        <v>5</v>
+      </c>
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>0</v>
+      </c>
+      <c r="K22">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.44247787610619471</v>
+      </c>
+      <c r="N22" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.2123893805309734E-2</v>
+      </c>
+      <c r="O22" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P22" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.4966887417218544</v>
+      </c>
+      <c r="Q22" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.66225165562913912</v>
+      </c>
+      <c r="R22" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.3112582781456956E-2</v>
+      </c>
+      <c r="S22" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T22" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>441</v>
+      </c>
+      <c r="U22" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.9205298013245033</v>
+      </c>
+      <c r="V22" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.9513274336283186</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C23" s="1">
+        <v>45750</v>
+      </c>
+      <c r="D23" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>331</v>
+      </c>
+      <c r="E23" s="3">
+        <v>164</v>
+      </c>
+      <c r="F23">
+        <v>29</v>
+      </c>
+      <c r="G23">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.17682926829268292</v>
+      </c>
+      <c r="N23" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.8292682926829267E-2</v>
+      </c>
+      <c r="O23" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>1.2195121951219513E-2</v>
+      </c>
+      <c r="P23" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.49546827794561932</v>
+      </c>
+      <c r="Q23" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.7613293051359523E-2</v>
+      </c>
+      <c r="R23" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>9.0634441087613302E-3</v>
+      </c>
+      <c r="S23" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>6.0422960725075529E-3</v>
+      </c>
+      <c r="T23" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>239</v>
+      </c>
+      <c r="U23" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.72205438066465255</v>
+      </c>
+      <c r="V23" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.4573170731707317</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="1">
+        <v>45932</v>
+      </c>
+      <c r="D24" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>149</v>
+      </c>
+      <c r="E24" s="3">
+        <v>123</v>
+      </c>
+      <c r="F24">
+        <v>12</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>9.7560975609756101E-2</v>
+      </c>
+      <c r="N24" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>8.130081300813009E-3</v>
+      </c>
+      <c r="O24" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>8.130081300813009E-3</v>
+      </c>
+      <c r="P24" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.82550335570469802</v>
+      </c>
+      <c r="Q24" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.0536912751677847E-2</v>
+      </c>
+      <c r="R24" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.7114093959731542E-3</v>
+      </c>
+      <c r="S24" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>6.7114093959731542E-3</v>
+      </c>
+      <c r="T24" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>154</v>
+      </c>
+      <c r="U24" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.0335570469798658</v>
+      </c>
+      <c r="V24" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.2520325203252032</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>46081</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="1">
+        <v>46034</v>
+      </c>
+      <c r="D25" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>47</v>
+      </c>
+      <c r="E25" s="3">
+        <v>86</v>
+      </c>
+      <c r="F25">
+        <v>24</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.27906976744186046</v>
+      </c>
+      <c r="N25" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.3255813953488372E-2</v>
+      </c>
+      <c r="O25" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P25" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.8297872340425532</v>
+      </c>
+      <c r="Q25" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.51063829787234039</v>
+      </c>
+      <c r="R25" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>4.2553191489361701E-2</v>
+      </c>
+      <c r="S25" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T25" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>140</v>
+      </c>
+      <c r="U25" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.978723404255319</v>
+      </c>
+      <c r="V25" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.6279069767441861</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="N8:N1048576 M1:M19">
+  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C25">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E8:E1048576 D1:D25">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F8:F1048576 E1:E25">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:G1048576 F1:F25">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H1:H25">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H8:H1048576 G1:G25">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N8:N1048576 M1:M25">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -2096,7 +2640,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O8:O1048576 N1:N19">
+  <conditionalFormatting sqref="O8:O1048576 N1:N25">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -2108,7 +2652,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8:Q1048576 O1:P19">
+  <conditionalFormatting sqref="P8:Q1048576 O1:P25">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -2120,67 +2664,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8:F1048576 E1:E19">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G8:G1048576 F1:F19">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H8:H1048576 G1:G19">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C19">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8:E1048576 D1:D19">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R8:R1048576 Q1:Q19">
+  <conditionalFormatting sqref="R8:R1048576 Q1:Q25">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -2192,7 +2676,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S8:S1048576 R1:R19">
+  <conditionalFormatting sqref="S8:S1048576 R1:R25">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -2204,7 +2688,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T8:T1048576 S1:S19">
+  <conditionalFormatting sqref="T8:T1048576 S1:S25">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -2216,7 +2700,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U8:U1048576 T1:T19">
+  <conditionalFormatting sqref="U8:U1048576 T1:T25">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -2228,7 +2712,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V8:V1048576 U1:U19">
+  <conditionalFormatting sqref="V8:V1048576 U1:U25">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -2240,20 +2724,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W8:W1048576 V1:V19">
+  <conditionalFormatting sqref="W8:W1048576 V1:V25">
     <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H19">
-    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
2026-03-06 NHL Scoreboard using Claude
</commit_message>
<xml_diff>
--- a/Python/Thingiverse/model_stats.xlsx
+++ b/Python/Thingiverse/model_stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Thingiverse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E9C4E2-ABA6-4FBC-85D3-9AA6DE276AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73043A7F-DF0D-46A8-86A9-5CD165CA681F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{AA65E66E-25AF-41FC-AF3D-E4037625FDAB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="28">
   <si>
     <t>Mammoth</t>
   </si>
@@ -208,8 +208,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V25" totalsRowShown="0">
-  <autoFilter ref="A1:V25" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V31" totalsRowShown="0">
+  <autoFilter ref="A1:V31" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
   <tableColumns count="22">
     <tableColumn id="22" xr3:uid="{B838C6CD-92E8-4070-81DB-2EDE900509A2}" name="Date"/>
     <tableColumn id="1" xr3:uid="{C06BFB11-D5FB-45F8-853C-B38F6CA36FF6}" name="Model"/>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC85C3B-1FD4-46FE-8A2F-07E281673B93}">
-  <dimension ref="A1:W25"/>
+  <dimension ref="A1:W31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
@@ -2555,8 +2555,482 @@
         <v>1.6279069767441861</v>
       </c>
     </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" s="1">
+        <v>45784</v>
+      </c>
+      <c r="D26" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>302</v>
+      </c>
+      <c r="E26" s="3">
+        <v>697</v>
+      </c>
+      <c r="F26">
+        <v>159</v>
+      </c>
+      <c r="G26">
+        <v>12</v>
+      </c>
+      <c r="H26">
+        <v>5</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.22812051649928264</v>
+      </c>
+      <c r="N26" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.721664275466284E-2</v>
+      </c>
+      <c r="O26" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>7.1736011477761836E-3</v>
+      </c>
+      <c r="P26" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.3079470198675498</v>
+      </c>
+      <c r="Q26" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.52649006622516559</v>
+      </c>
+      <c r="R26" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.9735099337748346E-2</v>
+      </c>
+      <c r="S26" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.6556291390728478E-2</v>
+      </c>
+      <c r="T26" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>1071</v>
+      </c>
+      <c r="U26" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.5463576158940397</v>
+      </c>
+      <c r="V26" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.5365853658536586</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1">
+        <v>45785</v>
+      </c>
+      <c r="D27" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>301</v>
+      </c>
+      <c r="E27" s="3">
+        <v>337</v>
+      </c>
+      <c r="F27">
+        <v>95</v>
+      </c>
+      <c r="G27">
+        <v>5</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.28189910979228489</v>
+      </c>
+      <c r="N27" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.483679525222552E-2</v>
+      </c>
+      <c r="O27" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>2.967359050445104E-3</v>
+      </c>
+      <c r="P27" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.1196013289036544</v>
+      </c>
+      <c r="Q27" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.31561461794019935</v>
+      </c>
+      <c r="R27" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>1.6611295681063124E-2</v>
+      </c>
+      <c r="S27" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>3.3222591362126247E-3</v>
+      </c>
+      <c r="T27" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>546</v>
+      </c>
+      <c r="U27" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.8139534883720929</v>
+      </c>
+      <c r="V27" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.6201780415430267</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2</v>
+      </c>
+      <c r="C28" s="1">
+        <v>45930</v>
+      </c>
+      <c r="D28" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>156</v>
+      </c>
+      <c r="E28" s="3">
+        <v>236</v>
+      </c>
+      <c r="F28">
+        <v>102</v>
+      </c>
+      <c r="G28">
+        <v>5</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.43220338983050849</v>
+      </c>
+      <c r="N28" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.1186440677966101E-2</v>
+      </c>
+      <c r="O28" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P28" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.5128205128205128</v>
+      </c>
+      <c r="Q28" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.65384615384615385</v>
+      </c>
+      <c r="R28" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.2051282051282048E-2</v>
+      </c>
+      <c r="S28" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T28" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>455</v>
+      </c>
+      <c r="U28" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.9166666666666665</v>
+      </c>
+      <c r="V28" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.9279661016949152</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B29" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="1">
+        <v>45750</v>
+      </c>
+      <c r="D29" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>336</v>
+      </c>
+      <c r="E29" s="3">
+        <v>167</v>
+      </c>
+      <c r="F29">
+        <v>31</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
+        <v>0</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.18562874251497005</v>
+      </c>
+      <c r="N29" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>5.9880239520958087E-3</v>
+      </c>
+      <c r="O29" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>5.9880239520958087E-3</v>
+      </c>
+      <c r="P29" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.49702380952380953</v>
+      </c>
+      <c r="Q29" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>9.2261904761904767E-2</v>
+      </c>
+      <c r="R29" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>2.976190476190476E-3</v>
+      </c>
+      <c r="S29" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>2.976190476190476E-3</v>
+      </c>
+      <c r="T29" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>236</v>
+      </c>
+      <c r="U29" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.70238095238095233</v>
+      </c>
+      <c r="V29" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.4131736526946108</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C30" s="1">
+        <v>45932</v>
+      </c>
+      <c r="D30" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>154</v>
+      </c>
+      <c r="E30" s="3">
+        <v>125</v>
+      </c>
+      <c r="F30">
+        <v>15</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>0</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.12</v>
+      </c>
+      <c r="N30" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="O30" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="P30" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.81168831168831168</v>
+      </c>
+      <c r="Q30" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>9.7402597402597407E-2</v>
+      </c>
+      <c r="R30" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.4935064935064939E-3</v>
+      </c>
+      <c r="S30" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>6.4935064935064939E-3</v>
+      </c>
+      <c r="T30" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>162</v>
+      </c>
+      <c r="U30" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.051948051948052</v>
+      </c>
+      <c r="V30" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.296</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="1">
+        <v>46034</v>
+      </c>
+      <c r="D31" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>52</v>
+      </c>
+      <c r="E31" s="3">
+        <v>96</v>
+      </c>
+      <c r="F31">
+        <v>27</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.28125</v>
+      </c>
+      <c r="N31" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="O31" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P31" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.8461538461538463</v>
+      </c>
+      <c r="Q31" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.51923076923076927</v>
+      </c>
+      <c r="R31" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.8461538461538464E-2</v>
+      </c>
+      <c r="S31" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T31" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>156</v>
+      </c>
+      <c r="U31" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3</v>
+      </c>
+      <c r="V31" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.625</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C25">
+  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C31">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -2568,7 +3042,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E8:E1048576 D1:D25">
+  <conditionalFormatting sqref="E8:E1048576 D1:D31">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -2580,7 +3054,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8:F1048576 E1:E25">
+  <conditionalFormatting sqref="F8:F1048576 E1:E31">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -2592,7 +3066,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8:G1048576 F1:F25">
+  <conditionalFormatting sqref="G8:G1048576 F1:F31">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -2604,7 +3078,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H25">
+  <conditionalFormatting sqref="H1:H31">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2616,7 +3090,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:H1048576 G1:G25">
+  <conditionalFormatting sqref="H8:H1048576 G1:G31">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -2628,7 +3102,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N8:N1048576 M1:M25">
+  <conditionalFormatting sqref="N8:N1048576 M1:M31">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -2640,7 +3114,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O8:O1048576 N1:N25">
+  <conditionalFormatting sqref="O8:O1048576 N1:N31">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -2652,7 +3126,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8:Q1048576 O1:P25">
+  <conditionalFormatting sqref="P8:Q1048576 O1:P31">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -2664,7 +3138,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R8:R1048576 Q1:Q25">
+  <conditionalFormatting sqref="R8:R1048576 Q1:Q31">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -2676,7 +3150,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S8:S1048576 R1:R25">
+  <conditionalFormatting sqref="S8:S1048576 R1:R31">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -2688,7 +3162,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T8:T1048576 S1:S25">
+  <conditionalFormatting sqref="T8:T1048576 S1:S31">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -2700,7 +3174,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U8:U1048576 T1:T25">
+  <conditionalFormatting sqref="U8:U1048576 T1:T31">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -2712,7 +3186,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V8:V1048576 U1:U25">
+  <conditionalFormatting sqref="V8:V1048576 U1:U31">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -2724,7 +3198,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W8:W1048576 V1:V25">
+  <conditionalFormatting sqref="W8:W1048576 V1:V31">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
2026-03-16 GamePredictions, New Dashboard, New Predctions Analysis
</commit_message>
<xml_diff>
--- a/Python/Thingiverse/model_stats.xlsx
+++ b/Python/Thingiverse/model_stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Thingiverse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73043A7F-DF0D-46A8-86A9-5CD165CA681F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D42A60-37D6-444F-AA94-4E207F978E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{AA65E66E-25AF-41FC-AF3D-E4037625FDAB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
   <si>
     <t>Mammoth</t>
   </si>
@@ -208,8 +208,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V31" totalsRowShown="0">
-  <autoFilter ref="A1:V31" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V37" totalsRowShown="0">
+  <autoFilter ref="A1:V37" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
   <tableColumns count="22">
     <tableColumn id="22" xr3:uid="{B838C6CD-92E8-4070-81DB-2EDE900509A2}" name="Date"/>
     <tableColumn id="1" xr3:uid="{C06BFB11-D5FB-45F8-853C-B38F6CA36FF6}" name="Model"/>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC85C3B-1FD4-46FE-8A2F-07E281673B93}">
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:W37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
@@ -3029,8 +3029,482 @@
         <v>1.625</v>
       </c>
     </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B32" t="s">
+        <v>0</v>
+      </c>
+      <c r="C32" s="1">
+        <v>45784</v>
+      </c>
+      <c r="D32" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>308</v>
+      </c>
+      <c r="E32" s="3">
+        <v>713</v>
+      </c>
+      <c r="F32">
+        <v>162</v>
+      </c>
+      <c r="G32">
+        <v>12</v>
+      </c>
+      <c r="H32">
+        <v>5</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
+      </c>
+      <c r="K32">
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.22720897615708274</v>
+      </c>
+      <c r="N32" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.6830294530154277E-2</v>
+      </c>
+      <c r="O32" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>7.0126227208976155E-3</v>
+      </c>
+      <c r="P32" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.3149350649350651</v>
+      </c>
+      <c r="Q32" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.52597402597402598</v>
+      </c>
+      <c r="R32" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.896103896103896E-2</v>
+      </c>
+      <c r="S32" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.6233766233766232E-2</v>
+      </c>
+      <c r="T32" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>1093</v>
+      </c>
+      <c r="U32" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.5487012987012987</v>
+      </c>
+      <c r="V32" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.5329593267882189</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" s="1">
+        <v>45785</v>
+      </c>
+      <c r="D33" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>307</v>
+      </c>
+      <c r="E33" s="3">
+        <v>341</v>
+      </c>
+      <c r="F33">
+        <v>96</v>
+      </c>
+      <c r="G33">
+        <v>5</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
+        <v>0</v>
+      </c>
+      <c r="L33">
+        <v>0</v>
+      </c>
+      <c r="M33" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.28152492668621704</v>
+      </c>
+      <c r="N33" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.466275659824047E-2</v>
+      </c>
+      <c r="O33" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>2.9325513196480938E-3</v>
+      </c>
+      <c r="P33" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.1107491856677525</v>
+      </c>
+      <c r="Q33" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.31270358306188922</v>
+      </c>
+      <c r="R33" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>1.6286644951140065E-2</v>
+      </c>
+      <c r="S33" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>3.2573289902280132E-3</v>
+      </c>
+      <c r="T33" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>552</v>
+      </c>
+      <c r="U33" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7980456026058631</v>
+      </c>
+      <c r="V33" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.6187683284457477</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" s="1">
+        <v>45930</v>
+      </c>
+      <c r="D34" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>162</v>
+      </c>
+      <c r="E34" s="3">
+        <v>242</v>
+      </c>
+      <c r="F34">
+        <v>102</v>
+      </c>
+      <c r="G34">
+        <v>5</v>
+      </c>
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34">
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <v>0</v>
+      </c>
+      <c r="L34">
+        <v>0</v>
+      </c>
+      <c r="M34" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.42148760330578511</v>
+      </c>
+      <c r="N34" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.0661157024793389E-2</v>
+      </c>
+      <c r="O34" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P34" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.4938271604938271</v>
+      </c>
+      <c r="Q34" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.62962962962962965</v>
+      </c>
+      <c r="R34" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.0864197530864196E-2</v>
+      </c>
+      <c r="S34" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T34" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>461</v>
+      </c>
+      <c r="U34" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.8456790123456792</v>
+      </c>
+      <c r="V34" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.9049586776859504</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="1">
+        <v>45750</v>
+      </c>
+      <c r="D35" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>342</v>
+      </c>
+      <c r="E35" s="3">
+        <v>168</v>
+      </c>
+      <c r="F35">
+        <v>31</v>
+      </c>
+      <c r="G35">
+        <v>3</v>
+      </c>
+      <c r="H35">
+        <v>2</v>
+      </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="M35" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.18452380952380953</v>
+      </c>
+      <c r="N35" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.7857142857142856E-2</v>
+      </c>
+      <c r="O35" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>1.1904761904761904E-2</v>
+      </c>
+      <c r="P35" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.49122807017543857</v>
+      </c>
+      <c r="Q35" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>9.0643274853801165E-2</v>
+      </c>
+      <c r="R35" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>8.771929824561403E-3</v>
+      </c>
+      <c r="S35" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>5.8479532163742687E-3</v>
+      </c>
+      <c r="T35" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>247</v>
+      </c>
+      <c r="U35" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="V35" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.4702380952380953</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B36" t="s">
+        <v>3</v>
+      </c>
+      <c r="C36" s="1">
+        <v>45932</v>
+      </c>
+      <c r="D36" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>160</v>
+      </c>
+      <c r="E36" s="3">
+        <v>126</v>
+      </c>
+      <c r="F36">
+        <v>15</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
+        <v>0</v>
+      </c>
+      <c r="L36">
+        <v>0</v>
+      </c>
+      <c r="M36" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.11904761904761904</v>
+      </c>
+      <c r="N36" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>7.9365079365079361E-3</v>
+      </c>
+      <c r="O36" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>7.9365079365079361E-3</v>
+      </c>
+      <c r="P36" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.78749999999999998</v>
+      </c>
+      <c r="Q36" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>9.375E-2</v>
+      </c>
+      <c r="R36" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>6.2500000000000003E-3</v>
+      </c>
+      <c r="S36" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>6.2500000000000003E-3</v>
+      </c>
+      <c r="T36" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>163</v>
+      </c>
+      <c r="U36" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.01875</v>
+      </c>
+      <c r="V36" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.2936507936507937</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>46092</v>
+      </c>
+      <c r="B37" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="1">
+        <v>46034</v>
+      </c>
+      <c r="D37" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>58</v>
+      </c>
+      <c r="E37" s="3">
+        <v>99</v>
+      </c>
+      <c r="F37">
+        <v>27</v>
+      </c>
+      <c r="G37">
+        <v>2</v>
+      </c>
+      <c r="H37">
+        <v>0</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="M37" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.27272727272727271</v>
+      </c>
+      <c r="N37" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.0202020202020204E-2</v>
+      </c>
+      <c r="O37" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P37" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.7068965517241379</v>
+      </c>
+      <c r="Q37" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.46551724137931033</v>
+      </c>
+      <c r="R37" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.4482758620689655E-2</v>
+      </c>
+      <c r="S37" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T37" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>159</v>
+      </c>
+      <c r="U37" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.7413793103448274</v>
+      </c>
+      <c r="V37" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.606060606060606</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C31">
+  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C37">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -3042,7 +3516,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E8:E1048576 D1:D31">
+  <conditionalFormatting sqref="E8:E1048576 D1:D37">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -3054,7 +3528,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8:F1048576 E1:E31">
+  <conditionalFormatting sqref="F8:F1048576 E1:E37">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -3066,7 +3540,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8:G1048576 F1:F31">
+  <conditionalFormatting sqref="G8:G1048576 F1:F37">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -3078,7 +3552,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H31">
+  <conditionalFormatting sqref="H1:H37">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -3090,7 +3564,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:H1048576 G1:G31">
+  <conditionalFormatting sqref="H8:H1048576 G1:G37">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -3102,7 +3576,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N8:N1048576 M1:M31">
+  <conditionalFormatting sqref="N8:N1048576 M1:M37">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -3114,7 +3588,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O8:O1048576 N1:N31">
+  <conditionalFormatting sqref="O8:O1048576 N1:N37">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -3126,7 +3600,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8:Q1048576 O1:P31">
+  <conditionalFormatting sqref="P8:Q1048576 O1:P37">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -3138,7 +3612,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R8:R1048576 Q1:Q31">
+  <conditionalFormatting sqref="R8:R1048576 Q1:Q37">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -3150,7 +3624,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S8:S1048576 R1:R31">
+  <conditionalFormatting sqref="S8:S1048576 R1:R37">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -3162,7 +3636,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T8:T1048576 S1:S31">
+  <conditionalFormatting sqref="T8:T1048576 S1:S37">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -3174,7 +3648,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U8:U1048576 T1:T31">
+  <conditionalFormatting sqref="U8:U1048576 T1:T37">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -3186,7 +3660,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V8:V1048576 U1:U31">
+  <conditionalFormatting sqref="V8:V1048576 U1:U37">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -3198,7 +3672,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W8:W1048576 V1:V31">
+  <conditionalFormatting sqref="W8:W1048576 V1:V37">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
2026-03-22 NHL Predictions update, added clinching scenarios, and edits to API reference examples
</commit_message>
<xml_diff>
--- a/Python/Thingiverse/model_stats.xlsx
+++ b/Python/Thingiverse/model_stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abrig\Documents\Coding_Practice\Python\Thingiverse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17D42A60-37D6-444F-AA94-4E207F978E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE1D7FE8-1FA4-4BA1-BCAC-59B416811F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{AA65E66E-25AF-41FC-AF3D-E4037625FDAB}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="28">
   <si>
     <t>Mammoth</t>
   </si>
@@ -208,8 +208,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V37" totalsRowShown="0">
-  <autoFilter ref="A1:V37" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}" name="Table1" displayName="Table1" ref="A1:V43" totalsRowShown="0">
+  <autoFilter ref="A1:V43" xr:uid="{83CFD035-DF42-4179-A65F-EE1B5D7828A5}"/>
   <tableColumns count="22">
     <tableColumn id="22" xr3:uid="{B838C6CD-92E8-4070-81DB-2EDE900509A2}" name="Date"/>
     <tableColumn id="1" xr3:uid="{C06BFB11-D5FB-45F8-853C-B38F6CA36FF6}" name="Model"/>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AC85C3B-1FD4-46FE-8A2F-07E281673B93}">
-  <dimension ref="A1:W37"/>
+  <dimension ref="A1:W43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
@@ -3503,8 +3503,482 @@
         <v>1.606060606060606</v>
       </c>
     </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B38" t="s">
+        <v>0</v>
+      </c>
+      <c r="C38" s="1">
+        <v>45784</v>
+      </c>
+      <c r="D38" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>315</v>
+      </c>
+      <c r="E38" s="3">
+        <v>733</v>
+      </c>
+      <c r="F38">
+        <v>167</v>
+      </c>
+      <c r="G38">
+        <v>13</v>
+      </c>
+      <c r="H38">
+        <v>5</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+      <c r="M38" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.22783083219645292</v>
+      </c>
+      <c r="N38" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.7735334242837655E-2</v>
+      </c>
+      <c r="O38" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>6.8212824010914054E-3</v>
+      </c>
+      <c r="P38" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>2.3269841269841272</v>
+      </c>
+      <c r="Q38" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.53015873015873016</v>
+      </c>
+      <c r="R38" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>4.1269841269841269E-2</v>
+      </c>
+      <c r="S38" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>1.5873015873015872E-2</v>
+      </c>
+      <c r="T38" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>1126</v>
+      </c>
+      <c r="U38" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>3.5746031746031748</v>
+      </c>
+      <c r="V38" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.5361527967257844</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1">
+        <v>45785</v>
+      </c>
+      <c r="D39" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>314</v>
+      </c>
+      <c r="E39" s="3">
+        <v>348</v>
+      </c>
+      <c r="F39">
+        <v>103</v>
+      </c>
+      <c r="G39">
+        <v>7</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
+        <v>0</v>
+      </c>
+      <c r="L39">
+        <v>0</v>
+      </c>
+      <c r="M39" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.29597701149425287</v>
+      </c>
+      <c r="N39" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.0114942528735632E-2</v>
+      </c>
+      <c r="O39" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>2.8735632183908046E-3</v>
+      </c>
+      <c r="P39" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.10828025477707</v>
+      </c>
+      <c r="Q39" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.32802547770700635</v>
+      </c>
+      <c r="R39" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>2.2292993630573247E-2</v>
+      </c>
+      <c r="S39" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>3.1847133757961785E-3</v>
+      </c>
+      <c r="T39" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>579</v>
+      </c>
+      <c r="U39" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.8439490445859872</v>
+      </c>
+      <c r="V39" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.6637931034482758</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B40" t="s">
+        <v>2</v>
+      </c>
+      <c r="C40" s="1">
+        <v>45930</v>
+      </c>
+      <c r="D40" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>169</v>
+      </c>
+      <c r="E40" s="3">
+        <v>246</v>
+      </c>
+      <c r="F40">
+        <v>103</v>
+      </c>
+      <c r="G40">
+        <v>5</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>0</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+      <c r="M40" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.41869918699186992</v>
+      </c>
+      <c r="N40" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>2.032520325203252E-2</v>
+      </c>
+      <c r="O40" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P40" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.455621301775148</v>
+      </c>
+      <c r="Q40" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.60946745562130178</v>
+      </c>
+      <c r="R40" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>2.9585798816568046E-2</v>
+      </c>
+      <c r="S40" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T40" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>467</v>
+      </c>
+      <c r="U40" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.7633136094674557</v>
+      </c>
+      <c r="V40" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.8983739837398375</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B41" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="1">
+        <v>45750</v>
+      </c>
+      <c r="D41" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>349</v>
+      </c>
+      <c r="E41" s="3">
+        <v>172</v>
+      </c>
+      <c r="F41">
+        <v>34</v>
+      </c>
+      <c r="G41">
+        <v>3</v>
+      </c>
+      <c r="H41">
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.19767441860465115</v>
+      </c>
+      <c r="N41" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.7441860465116279E-2</v>
+      </c>
+      <c r="O41" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>1.1627906976744186E-2</v>
+      </c>
+      <c r="P41" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.49283667621776506</v>
+      </c>
+      <c r="Q41" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>9.7421203438395415E-2</v>
+      </c>
+      <c r="R41" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>8.5959885386819486E-3</v>
+      </c>
+      <c r="S41" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>5.7306590257879654E-3</v>
+      </c>
+      <c r="T41" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>257</v>
+      </c>
+      <c r="U41" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>0.73638968481375355</v>
+      </c>
+      <c r="V41" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.4941860465116279</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B42" t="s">
+        <v>3</v>
+      </c>
+      <c r="C42" s="1">
+        <v>45932</v>
+      </c>
+      <c r="D42" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>167</v>
+      </c>
+      <c r="E42" s="3">
+        <v>131</v>
+      </c>
+      <c r="F42">
+        <v>15</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <v>0</v>
+      </c>
+      <c r="K42">
+        <v>0</v>
+      </c>
+      <c r="L42">
+        <v>0</v>
+      </c>
+      <c r="M42" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.11450381679389313</v>
+      </c>
+      <c r="N42" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>7.6335877862595417E-3</v>
+      </c>
+      <c r="O42" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>7.6335877862595417E-3</v>
+      </c>
+      <c r="P42" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>0.78443113772455086</v>
+      </c>
+      <c r="Q42" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>8.9820359281437126E-2</v>
+      </c>
+      <c r="R42" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>5.9880239520958087E-3</v>
+      </c>
+      <c r="S42" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>5.9880239520958087E-3</v>
+      </c>
+      <c r="T42" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>168</v>
+      </c>
+      <c r="U42" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>1.0059880239520957</v>
+      </c>
+      <c r="V42" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.282442748091603</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B43" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="1">
+        <v>46034</v>
+      </c>
+      <c r="D43" s="2">
+        <f>Table1[[#This Row],[Date]]-Table1[[#This Row],[Published]]</f>
+        <v>65</v>
+      </c>
+      <c r="E43" s="3">
+        <v>101</v>
+      </c>
+      <c r="F43">
+        <v>28</v>
+      </c>
+      <c r="G43">
+        <v>2</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43">
+        <v>0</v>
+      </c>
+      <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Views]]</f>
+        <v>0.27722772277227725</v>
+      </c>
+      <c r="N43" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Views]]</f>
+        <v>1.9801980198019802E-2</v>
+      </c>
+      <c r="O43" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Views]]</f>
+        <v>0</v>
+      </c>
+      <c r="P43" s="4">
+        <f>Table1[[#This Row],[Views]]/Table1[[#This Row],[Age]]</f>
+        <v>1.5538461538461539</v>
+      </c>
+      <c r="Q43" s="4">
+        <f>Table1[[#This Row],[Downloads]]/Table1[[#This Row],[Age]]</f>
+        <v>0.43076923076923079</v>
+      </c>
+      <c r="R43" s="4">
+        <f>Table1[[#This Row],[Likes]]/Table1[[#This Row],[Age]]</f>
+        <v>3.0769230769230771E-2</v>
+      </c>
+      <c r="S43" s="4">
+        <f>Table1[[#This Row],[Collects]]/Table1[[#This Row],[Age]]</f>
+        <v>0</v>
+      </c>
+      <c r="T43" s="4">
+        <f>(4*Table1[[#This Row],[Collects]])+(3*Table1[[#This Row],[Likes]])+(2*Table1[[#This Row],[Downloads]])+Table1[[#This Row],[Views]]</f>
+        <v>163</v>
+      </c>
+      <c r="U43" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Age]]</f>
+        <v>2.5076923076923077</v>
+      </c>
+      <c r="V43" s="4">
+        <f>Table1[[#This Row],[Score]]/Table1[[#This Row],[Views]]</f>
+        <v>1.613861386138614</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C37">
+  <conditionalFormatting sqref="C1:D7 D8:E1048576 C8:C43">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -3516,7 +3990,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E8:E1048576 D1:D37">
+  <conditionalFormatting sqref="E8:E1048576 D1:D43">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -3528,7 +4002,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8:F1048576 E1:E37">
+  <conditionalFormatting sqref="F8:F1048576 E1:E43">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -3540,7 +4014,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8:G1048576 F1:F37">
+  <conditionalFormatting sqref="G8:G1048576 F1:F43">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -3552,7 +4026,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H1:H37">
+  <conditionalFormatting sqref="H1:H43">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -3564,7 +4038,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8:H1048576 G1:G37">
+  <conditionalFormatting sqref="H8:H1048576 G1:G43">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -3576,7 +4050,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N8:N1048576 M1:M37">
+  <conditionalFormatting sqref="N8:N1048576 M1:M43">
     <cfRule type="colorScale" priority="16">
       <colorScale>
         <cfvo type="min"/>
@@ -3588,7 +4062,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O8:O1048576 N1:N37">
+  <conditionalFormatting sqref="O8:O1048576 N1:N43">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -3600,7 +4074,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8:Q1048576 O1:P37">
+  <conditionalFormatting sqref="P8:Q1048576 O1:P43">
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="min"/>
@@ -3612,7 +4086,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R8:R1048576 Q1:Q37">
+  <conditionalFormatting sqref="R8:R1048576 Q1:Q43">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -3624,7 +4098,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S8:S1048576 R1:R37">
+  <conditionalFormatting sqref="S8:S1048576 R1:R43">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -3636,7 +4110,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T8:T1048576 S1:S37">
+  <conditionalFormatting sqref="T8:T1048576 S1:S43">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -3648,7 +4122,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U8:U1048576 T1:T37">
+  <conditionalFormatting sqref="U8:U1048576 T1:T43">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -3660,7 +4134,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V8:V1048576 U1:U37">
+  <conditionalFormatting sqref="V8:V1048576 U1:U43">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -3672,7 +4146,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W8:W1048576 V1:V37">
+  <conditionalFormatting sqref="W8:W1048576 V1:V43">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>